<commit_message>
docs: document item scope and add it to the sample workbook Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SampleChecklist.xlsx
+++ b/SampleChecklist.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -732,6 +732,48 @@
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DA Consent (NOD document)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>F02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BCA Report</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -894,7 +936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -908,6 +950,11 @@
           <t>Name</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -920,6 +967,7 @@
           <t>Architectural</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -932,6 +980,7 @@
           <t>Structural</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -942,6 +991,24 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>Electrical</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>project</t>
         </is>
       </c>
     </row>

</xml_diff>